<commit_message>
Excel: eliminar sheets Formulas y Backtest
</commit_message>
<xml_diff>
--- a/Resultados/proyeccion_costos.xlsx
+++ b/Resultados/proyeccion_costos.xlsx
@@ -1,16 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyeccion" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backtest" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Proyeccion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metodo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1043,308 +1041,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="0010b981"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Backtest — Comparacion de Metodos (MAE en $)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Datos mensuales 2010-2023 (164 meses). Rolling origin: cada mes usa solo datos hasta t-1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Materia Prima</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Naive</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>SMA(3)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>SMA(6)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Mejor metodo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="n">
-        <v>4.476343056530727</v>
-      </c>
-      <c r="C5" s="9" t="n">
-        <v>6.192249395980797</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>7.881408872149457</v>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Naive</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="n">
-        <v>24.27811951700829</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>38.26835279194373</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>49.50071275361793</v>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>Naive</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n">
-        <v>78.12894469283859</v>
-      </c>
-      <c r="C7" s="9" t="n">
-        <v>111.0859647235454</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>148.7434700432091</v>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Naive</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Conclusinn: Naive gana en 3/3 materias primas. Es el metodo mas consistente y el unico que nunca pierde.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A9:E9"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="008b5cf6"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Formulas Paso a Paso</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Reproduce la proyeccion manualmente sin depender del agente</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Paso</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Ejemplo con datos actuales</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>1. Obtener Y, Z</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Promedio del ultimo mes de datos historicos</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>Y = $555.33, Z = $2142.52</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>2. Calcular Eq1 diario</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>Eq1 = 0.8182 * Y + 5.49</t>
-        </is>
-      </c>
-      <c r="C6" s="23">
-        <f> 0.8182*555.33 + 5.49 = $459.87</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>3. Calcular Eq2 diario</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Eq2 = 0.3551*Y + 0.3368*Z + 6.49</t>
-        </is>
-      </c>
-      <c r="C7" s="21">
-        <f> ... = $925.29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t>4. Costo mensual Eq1</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>Eq1_diario * 22 dias habiles</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>$459.87 * 22 = $10,117.16</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>5. Costo mensual Eq2</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>Eq2_diario * 22 dias habiles</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>$925.29 * 22 = $20,356.45</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>6. IC 95% mes N</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>1.96 * sigma * sqrt(N)</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>Mes 1 Eq1: 1.96*4.69*sqrt(1) = +-$9.19</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>7. IC acumulado N meses</t>
-        </is>
-      </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>1.96 * sigma * sqrt(N) * 22</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>3m Eq1: 1.96*4.69*sqrt(3)*22 = +-$350.19</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>